<commit_message>
update code BE fr server
</commit_message>
<xml_diff>
--- a/BE/HVDS_BE/data.xlsx
+++ b/BE/HVDS_BE/data.xlsx
@@ -4,13 +4,14 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="18350" windowHeight="6800" activeTab="3"/>
+    <workbookView windowWidth="18350" windowHeight="6800" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Location" sheetId="1" r:id="rId1"/>
     <sheet name="Camera" sheetId="2" r:id="rId2"/>
     <sheet name="ViolationStatus" sheetId="3" r:id="rId3"/>
     <sheet name="Account" sheetId="4" r:id="rId4"/>
+    <sheet name="Citizen" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="118">
   <si>
     <t>name</t>
   </si>
@@ -257,15 +258,6 @@
     <t>email</t>
   </si>
   <si>
-    <t>admin</t>
-  </si>
-  <si>
-    <t>Admin</t>
-  </si>
-  <si>
-    <t>admin@gmail.com</t>
-  </si>
-  <si>
     <t>supervisor</t>
   </si>
   <si>
@@ -279,6 +271,120 @@
   </si>
   <si>
     <t>supervisor2@gmail.com</t>
+  </si>
+  <si>
+    <t>citizen_identity_id</t>
+  </si>
+  <si>
+    <t>full_name</t>
+  </si>
+  <si>
+    <t>phone_number</t>
+  </si>
+  <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>dob</t>
+  </si>
+  <si>
+    <t>place_of_birth</t>
+  </si>
+  <si>
+    <t>gender</t>
+  </si>
+  <si>
+    <t>issue_date</t>
+  </si>
+  <si>
+    <t>place_of_issue</t>
+  </si>
+  <si>
+    <t>nationality</t>
+  </si>
+  <si>
+    <t>0473483788</t>
+  </si>
+  <si>
+    <t>Hoàng Ngọc Xuân Nguyên</t>
+  </si>
+  <si>
+    <t>0777215598</t>
+  </si>
+  <si>
+    <t>hoangnguyen01022003@gmail.com</t>
+  </si>
+  <si>
+    <t>Hồ Chí Minh</t>
+  </si>
+  <si>
+    <t>female</t>
+  </si>
+  <si>
+    <t>Cục trưởng Cục Cảnh sát</t>
+  </si>
+  <si>
+    <t>Vietnam</t>
+  </si>
+  <si>
+    <t>0503837867</t>
+  </si>
+  <si>
+    <t>Đặng Thị Lệ Chi</t>
+  </si>
+  <si>
+    <t>0333690079</t>
+  </si>
+  <si>
+    <t>chidtl79@gmail.com</t>
+  </si>
+  <si>
+    <t>Bình ĐỊnh</t>
+  </si>
+  <si>
+    <t>0376321983</t>
+  </si>
+  <si>
+    <t>Nguyễn Sơn Tùng</t>
+  </si>
+  <si>
+    <t>0335955790</t>
+  </si>
+  <si>
+    <t>nstung463@gmail.com</t>
+  </si>
+  <si>
+    <t>Lâm Đồng</t>
+  </si>
+  <si>
+    <t>male</t>
+  </si>
+  <si>
+    <t>0232354532</t>
+  </si>
+  <si>
+    <t>Lê Huy Hoàn</t>
+  </si>
+  <si>
+    <t>0935359107</t>
+  </si>
+  <si>
+    <t>hoanlh@gmail.com</t>
+  </si>
+  <si>
+    <t>0324343532</t>
+  </si>
+  <si>
+    <t>Nguyễn Trung Kiên</t>
+  </si>
+  <si>
+    <t>0866140558</t>
+  </si>
+  <si>
+    <t>kien.nguyentrung1699@gmail.com</t>
+  </si>
+  <si>
+    <t>Bình Định</t>
   </si>
 </sst>
 </file>
@@ -894,14 +1000,20 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="58" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1886,8 +1998,8 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="4"/>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="14.6363636363636" customWidth="1"/>
     <col min="2" max="2" width="17.1818181818182" customWidth="1"/>
@@ -1937,37 +2049,264 @@
         <v>123</v>
       </c>
       <c r="C3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>80</v>
-      </c>
       <c r="E3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>81</v>
-      </c>
-      <c r="B4">
-        <v>123</v>
-      </c>
-      <c r="C4" t="s">
-        <v>79</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="E4" t="s">
         <v>42</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" display="admin@gmail.com"/>
-    <hyperlink ref="D3" r:id="rId2" display="supervisor@gmail.com"/>
-    <hyperlink ref="D4" r:id="rId3" display="supervisor2@gmail.com" tooltip="mailto:supervisor2@gmail.com"/>
+    <hyperlink ref="D2" r:id="rId1" display="supervisor@gmail.com"/>
+    <hyperlink ref="D3" r:id="rId2" display="supervisor2@gmail.com" tooltip="mailto:supervisor2@gmail.com"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="5"/>
+  <cols>
+    <col min="1" max="1" width="17.5454545454545" customWidth="1"/>
+    <col min="2" max="2" width="24.4545454545455" customWidth="1"/>
+    <col min="3" max="3" width="15.1818181818182" customWidth="1"/>
+    <col min="4" max="4" width="14.8181818181818" customWidth="1"/>
+    <col min="5" max="5" width="17.5454545454545" customWidth="1"/>
+    <col min="6" max="6" width="10.4545454545455" customWidth="1"/>
+    <col min="7" max="7" width="17.1818181818182" customWidth="1"/>
+    <col min="8" max="8" width="17" customWidth="1"/>
+    <col min="10" max="10" width="10.5454545454545" customWidth="1"/>
+    <col min="11" max="11" width="14.3636363636364" customWidth="1"/>
+    <col min="12" max="12" width="10.4545454545455" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1" t="s">
+        <v>84</v>
+      </c>
+      <c r="H1" t="s">
+        <v>85</v>
+      </c>
+      <c r="I1" t="s">
+        <v>86</v>
+      </c>
+      <c r="J1" t="s">
+        <v>87</v>
+      </c>
+      <c r="K1" t="s">
+        <v>88</v>
+      </c>
+      <c r="L1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F2" t="s">
+        <v>65</v>
+      </c>
+      <c r="G2" s="2">
+        <v>37623</v>
+      </c>
+      <c r="H2" t="s">
+        <v>94</v>
+      </c>
+      <c r="I2" t="s">
+        <v>95</v>
+      </c>
+      <c r="K2" t="s">
+        <v>96</v>
+      </c>
+      <c r="L2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="E3" t="s">
+        <v>102</v>
+      </c>
+      <c r="F3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G3" s="2">
+        <v>37624</v>
+      </c>
+      <c r="H3" t="s">
+        <v>102</v>
+      </c>
+      <c r="I3" t="s">
+        <v>95</v>
+      </c>
+      <c r="K3" t="s">
+        <v>96</v>
+      </c>
+      <c r="L3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E4" t="s">
+        <v>107</v>
+      </c>
+      <c r="F4" t="s">
+        <v>65</v>
+      </c>
+      <c r="G4" s="2">
+        <v>37625</v>
+      </c>
+      <c r="H4" t="s">
+        <v>107</v>
+      </c>
+      <c r="I4" t="s">
+        <v>108</v>
+      </c>
+      <c r="K4" t="s">
+        <v>96</v>
+      </c>
+      <c r="L4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E5" t="s">
+        <v>94</v>
+      </c>
+      <c r="F5" t="s">
+        <v>65</v>
+      </c>
+      <c r="G5" s="2">
+        <v>37626</v>
+      </c>
+      <c r="H5" t="s">
+        <v>94</v>
+      </c>
+      <c r="I5" t="s">
+        <v>108</v>
+      </c>
+      <c r="K5" t="s">
+        <v>96</v>
+      </c>
+      <c r="L5" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B6" t="s">
+        <v>114</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="E6" t="s">
+        <v>117</v>
+      </c>
+      <c r="F6" t="s">
+        <v>65</v>
+      </c>
+      <c r="G6" s="2">
+        <v>37627</v>
+      </c>
+      <c r="H6" t="s">
+        <v>117</v>
+      </c>
+      <c r="I6" t="s">
+        <v>108</v>
+      </c>
+      <c r="K6" t="s">
+        <v>96</v>
+      </c>
+      <c r="L6" t="s">
+        <v>97</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" display="hoangnguyen01022003@gmail.com"/>
+    <hyperlink ref="D3" r:id="rId2" display="chidtl79@gmail.com"/>
+    <hyperlink ref="D4" r:id="rId3" display="nstung463@gmail.com"/>
+    <hyperlink ref="D6" r:id="rId4" display="kien.nguyentrung1699@gmail.com"/>
+    <hyperlink ref="D5" r:id="rId5" display="hoanlh@gmail.com"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>